<commit_message>
Pedido livre de violência contra pessoa idosa e primeira sincronização com a planilha Google
- Novo tema violidoso: frases como "avó apanhando", "idoso abandonado" ou
  "fica com a aposentadoria" ligam a situação violIdoso e a faixa de urgência.
- Bloco dados-planilha preenchido a partir da planilha: 56 serviços passam a
  mostrar "Conferido em" ou "Confirme antes de enviar a pessoa".
- CLAUDE.md registra o ID da planilha oficial.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014i5gioXTJeGHtBeLGKbgmY
</commit_message>
<xml_diff>
--- a/dados/banco-de-dados-encaminha.xlsx
+++ b/dados/banco-de-dados-encaminha.xlsx
@@ -233,7 +233,7 @@
   <commentList>
     <comment ref="A1" authorId="0" shapeId="0">
       <text>
-        <t>Fonte: Encaminha Goiânia, index.html (commit aead8b5), 23 linhas, exportado em 08/10/2026. Exportado por Claude. Detalhes na aba Fontes.</t>
+        <t>Fonte: Encaminha Goiânia, index.html (commit aead8b5), 24 linhas, exportado em 08/10/2026. Exportado por Claude. Detalhes na aba Fontes.</t>
       </text>
     </comment>
   </commentList>
@@ -12610,7 +12610,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G24"/>
+  <dimension ref="A1:G25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -13168,22 +13168,22 @@
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
         <is>
-          <t>discriminacao</t>
+          <t>violidoso</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>Discriminação: racismo, xenofobia, intolerância religiosa, LGBTfobia</t>
+          <t>Violência, abandono ou exploração de pessoa idosa ou com deficiência</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>racismo, racista, injuria racial, ofensa racial, preconceito, discrimina, xenofob, por ser nordestin, por ser estrangeir, por ser venezuelan, por ser haitian, volta pro seu pais, homofobia, homofob, transfobia, lgbtfobia, intolerancia religiosa, racismo religioso, atacaram o terreiro, ataque ao terreiro, invadiram o terreiro, por ser do candomble, por ser da umbanda, por causa da religiao, por causa da minha religiao, perseguido pela religiao, perseguida pela religiao, por ser evangelic, por ser catolic, por ser espirita, por ser muculman, por ser judeu, por ser judia, macumbeir, chutaram a imagem, capacitismo, capacitista, idadismo, etarismo, xingou de macaco</t>
+          <t>violencia contra idoso, violencia contra idosa, violencia contra o idoso, violencia contra a idosa, violencia contra pessoa idosa, violencia contra a pessoa idosa, violencia contra pessoa com deficiencia, violencia contra a pessoa com deficiencia, idoso apanha, idosa apanha, avo apanha, avo esta apanhando, avo ta apanhando, bate no idoso, bate na idosa, bate no avo, bate na avo, bateu no avo, bateu na avo, batendo no avo, batendo na avo, agride o idoso, agride a idosa, agrediu o idoso, agrediu a idosa, agressao ao idoso, agressao a idosa, maus tratos ao idoso, maus tratos a idosa, maus tratos contra idoso, maus tratos contra a pessoa idosa, maus tratos a pessoa com deficiencia, idoso sofrendo maus, idosa sofrendo maus, idoso sofrendo violencia, idosa sofrendo violencia, idoso maltratad, idosa maltratad, maltrata o idoso, maltrata a idosa, maltrata o avo, maltrata a avo, idoso abandonad, idosa abandonad, abandono de idoso, abandono do idoso, abandono da idosa, idoso largad, idosa largad, idoso negligenciad, idosa negligenciad, negligencia com idoso, negligencia com o idoso, negligencia com a idosa, idoso trancad, idosa trancad, pega o cartao do aposentad, pegam o cartao do aposentad, toma o cartao do aposentad, fica com o cartao do aposentad, pega a aposentadoria, pegam a aposentadoria, toma a aposentadoria, fica com a aposentadoria, fica com o dinheiro da aposentadoria, fica com o dinheiro do idoso, exploracao financeira, emprestimo no nome do idoso, emprestimo no nome da idosa, emprestimo no nome do avo, emprestimo no nome da avo</t>
         </is>
       </c>
       <c r="D18" s="6" t="inlineStr">
         <is>
-          <t>discrim</t>
+          <t>violIdoso</t>
         </is>
       </c>
       <c r="E18" s="3" t="inlineStr"/>
@@ -13193,21 +13193,46 @@
     <row r="19">
       <c r="A19" s="6" t="inlineStr">
         <is>
+          <t>discriminacao</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>Discriminação: racismo, xenofobia, intolerância religiosa, LGBTfobia</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>racismo, racista, injuria racial, ofensa racial, preconceito, discrimina, xenofob, por ser nordestin, por ser estrangeir, por ser venezuelan, por ser haitian, volta pro seu pais, homofobia, homofob, transfobia, lgbtfobia, intolerancia religiosa, racismo religioso, atacaram o terreiro, ataque ao terreiro, invadiram o terreiro, por ser do candomble, por ser da umbanda, por causa da religiao, por causa da minha religiao, perseguido pela religiao, perseguida pela religiao, por ser evangelic, por ser catolic, por ser espirita, por ser muculman, por ser judeu, por ser judia, macumbeir, chutaram a imagem, capacitismo, capacitista, idadismo, etarismo, xingou de macaco</t>
+        </is>
+      </c>
+      <c r="D19" s="6" t="inlineStr">
+        <is>
+          <t>discrim</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr"/>
+      <c r="F19" s="6" t="inlineStr"/>
+      <c r="G19" s="3" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="6" t="inlineStr">
+        <is>
           <t>trans</t>
         </is>
       </c>
-      <c r="B19" s="3" t="inlineStr">
+      <c r="B20" s="3" t="inlineStr">
         <is>
           <t>Pessoa trans: saúde e documentos</t>
         </is>
       </c>
-      <c r="C19" s="3" t="inlineStr">
+      <c r="C20" s="3" t="inlineStr">
         <is>
           <t>pessoa trans, mulher trans, homem trans, menina trans, menino trans, transexual, travesti, transgenero, hormonizacao, nome social, mudar o nome, redesignacao</t>
         </is>
       </c>
-      <c r="D19" s="6" t="inlineStr"/>
-      <c r="E19" s="3" t="inlineStr">
+      <c r="D20" s="6" t="inlineStr"/>
+      <c r="E20" s="3" t="inlineStr">
         <is>
           <t>Saúde: pedir na UBS o encaminhamento para o Ambulatório TX do HGG (hormonização, psicologia, cirurgias). Maiores de 18 em Goiânia também podem procurar o Transviver.
 Nome social: pode ser usado no SUS, na escola e no CadÚnico, sem mudar documento.
@@ -13215,31 +13240,31 @@
 Violência ou discriminação: Deacri e Disque 100.</t>
         </is>
       </c>
-      <c r="F19" s="6" t="inlineStr">
+      <c r="F20" s="6" t="inlineStr">
         <is>
           <t>hgg-tx, transviver, deacri, dpe</t>
         </is>
       </c>
-      <c r="G19" s="3" t="inlineStr"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="6" t="inlineStr">
+      <c r="G20" s="3" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="6" t="inlineStr">
         <is>
           <t>migrante</t>
         </is>
       </c>
-      <c r="B20" s="3" t="inlineStr">
+      <c r="B21" s="3" t="inlineStr">
         <is>
           <t>Migrantes e refugiados</t>
         </is>
       </c>
-      <c r="C20" s="3" t="inlineStr">
+      <c r="C21" s="3" t="inlineStr">
         <is>
           <t>migrante, imigrante, refugiad, venezuelan, haitian, estrangeir, refugio, sem documento brasileiro</t>
         </is>
       </c>
-      <c r="D20" s="6" t="inlineStr"/>
-      <c r="E20" s="3" t="inlineStr">
+      <c r="D21" s="6" t="inlineStr"/>
+      <c r="E21" s="3" t="inlineStr">
         <is>
           <t>O SUS atende sem exigir documento brasileiro. A criança tem direito à matrícula na escola.
 CadÚnico e benefícios: pode se cadastrar com a Carteira de Registro Nacional Migratório (CRNM) ou o protocolo de refúgio, no CRAS.
@@ -13248,31 +13273,31 @@
 Sofreu xenofobia: é crime (Lei 7.716/1989). Registrar na Deacri ou em qualquer delegacia, ou pelo Disque 100.</t>
         </is>
       </c>
-      <c r="F20" s="6" t="inlineStr">
+      <c r="F21" s="6" t="inlineStr">
         <is>
           <t>pastoral-migrantes, deacri, 100, 121</t>
         </is>
       </c>
-      <c r="G20" s="3" t="inlineStr"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="6" t="inlineStr">
+      <c r="G21" s="3" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="6" t="inlineStr">
         <is>
           <t>egresso</t>
         </is>
       </c>
-      <c r="B21" s="3" t="inlineStr">
+      <c r="B22" s="3" t="inlineStr">
         <is>
           <t>Saiu do sistema prisional (egresso) e família</t>
         </is>
       </c>
-      <c r="C21" s="3" t="inlineStr">
+      <c r="C22" s="3" t="inlineStr">
         <is>
           <t>egresso, saiu da prisao, saiu da cadeia, ex-detento, ex detento, presidiario, tornozeleira, liberdade condicional, foi preso, esta preso, presidio</t>
         </is>
       </c>
-      <c r="D21" s="6" t="inlineStr"/>
-      <c r="E21" s="3" t="inlineStr">
+      <c r="D22" s="6" t="inlineStr"/>
+      <c r="E22" s="3" t="inlineStr">
         <is>
           <t>Escritório Social (Goiânia): documentos, trabalho, estudo e acesso a políticas sociais para egressos e famílias. Atendimento voluntário.
 Família de pessoa presa: auxílio-reclusão no INSS, se a pessoa contribuía (Meu INSS ou 135).
@@ -13280,31 +13305,31 @@
 Dúvidas sobre a pena ou o processo: Defensoria Pública.</t>
         </is>
       </c>
-      <c r="F21" s="6" t="inlineStr">
+      <c r="F22" s="6" t="inlineStr">
         <is>
           <t>escritorio-social, dpe, 135</t>
         </is>
       </c>
-      <c r="G21" s="3" t="inlineStr"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="6" t="inlineStr">
+      <c r="G22" s="3" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="6" t="inlineStr">
         <is>
           <t>cancer</t>
         </is>
       </c>
-      <c r="B22" s="3" t="inlineStr">
+      <c r="B23" s="3" t="inlineStr">
         <is>
           <t>Câncer: diagnóstico e tratamento</t>
         </is>
       </c>
-      <c r="C22" s="3" t="inlineStr">
+      <c r="C23" s="3" t="inlineStr">
         <is>
           <t>cancer, tumor, quimioterapia, radioterapia, oncolog, biopsia, nodulo, metastase</t>
         </is>
       </c>
-      <c r="D22" s="6" t="inlineStr"/>
-      <c r="E22" s="3" t="inlineStr">
+      <c r="D23" s="6" t="inlineStr"/>
+      <c r="E23" s="3" t="inlineStr">
         <is>
           <t>Pela lei, exames para confirmar câncer devem sair em até 30 dias (Lei 13.896/2019) e o tratamento no SUS deve começar em até 60 dias do diagnóstico (Lei 12.732/2012).
 O encaminhamento sai da UBS ou do médico, pela regulação. Em Goiânia, a referência é o Hospital Araújo Jorge; também o HC-UFG.
@@ -13313,31 +13338,31 @@
 Transporte e hospedagem para quem vem do interior: pedir o Tratamento Fora de Domicílio (TFD) na Secretaria de Saúde do município.</t>
         </is>
       </c>
-      <c r="F22" s="6" t="inlineStr">
+      <c r="F23" s="6" t="inlineStr">
         <is>
           <t>araujo-jorge, hc-ufg, 136, dpe</t>
         </is>
       </c>
-      <c r="G22" s="3" t="inlineStr"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="6" t="inlineStr">
+      <c r="G23" s="3" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="6" t="inlineStr">
         <is>
           <t>trafico</t>
         </is>
       </c>
-      <c r="B23" s="3" t="inlineStr">
+      <c r="B24" s="3" t="inlineStr">
         <is>
           <t>Tráfico de pessoas e trabalho escravo</t>
         </is>
       </c>
-      <c r="C23" s="3" t="inlineStr">
+      <c r="C24" s="3" t="inlineStr">
         <is>
           <t>trafico de pessoas, trabalho escravo, escravidao, proposta de emprego no exterior, retiveram o passaporte, sem salario, nao deixam sair</t>
         </is>
       </c>
-      <c r="D23" s="6" t="inlineStr"/>
-      <c r="E23" s="3" t="inlineStr">
+      <c r="D24" s="6" t="inlineStr"/>
+      <c r="E24" s="3" t="inlineStr">
         <is>
           <t>Risco agora: 190.
 Denunciar pelo Disque 100 (24h, também pelo WhatsApp (61) 99611-0100) ou pelo Ligue 180. As denúncias de trabalho escravo seguem para a fiscalização do Ministério do Trabalho.
@@ -13345,39 +13370,39 @@
 Proposta de emprego no exterior boa demais, com passagem paga e documento retido: sinal de alerta.</t>
         </is>
       </c>
-      <c r="F23" s="6" t="inlineStr">
+      <c r="F24" s="6" t="inlineStr">
         <is>
           <t>100, 180, mpt</t>
         </is>
       </c>
-      <c r="G23" s="3" t="inlineStr"/>
-    </row>
-    <row r="24">
-      <c r="A24" s="6" t="inlineStr">
+      <c r="G24" s="3" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="6" t="inlineStr">
         <is>
           <t>dentista</t>
         </is>
       </c>
-      <c r="B24" s="3" t="inlineStr">
+      <c r="B25" s="3" t="inlineStr">
         <is>
           <t>Dentista</t>
         </is>
       </c>
-      <c r="C24" s="3" t="inlineStr">
+      <c r="C25" s="3" t="inlineStr">
         <is>
           <t>dente, dentista, odonto, dentadura, protese dentaria</t>
         </is>
       </c>
-      <c r="D24" s="6" t="inlineStr"/>
-      <c r="E24" s="3" t="inlineStr">
+      <c r="D25" s="6" t="inlineStr"/>
+      <c r="E25" s="3" t="inlineStr">
         <is>
           <t>Primeira consulta na UBS, com a equipe de saúde bucal.
 Tratamento especializado (canal, prótese, cirurgia): a UBS encaminha ao Centro de Especialidades Odontológicas (CEO).
 Dor forte ou rosto inchado: UPA ou CAIS 24h.</t>
         </is>
       </c>
-      <c r="F24" s="6" t="inlineStr"/>
-      <c r="G24" s="3" t="inlineStr"/>
+      <c r="F25" s="6" t="inlineStr"/>
+      <c r="G25" s="3" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -14591,7 +14616,7 @@
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
         <is>
-          <t>Temas!A1:G24</t>
+          <t>Temas!A1:G25</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
@@ -14622,7 +14647,7 @@
       </c>
       <c r="H4" s="6" t="inlineStr"/>
       <c r="I4" s="6" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="J4" s="3" t="inlineStr">
         <is>

</xml_diff>